<commit_message>
update feature importance +-sign
</commit_message>
<xml_diff>
--- a/src/attributions/attributions_ig_traj_100.xlsx
+++ b/src/attributions/attributions_ig_traj_100.xlsx
@@ -2140,19 +2140,19 @@
         <v>0</v>
       </c>
       <c r="B4" t="n">
-        <v>0.5528775001402585</v>
+        <v>0.5372669367838552</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="D4" t="n">
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>-0.01453760429325892</v>
+        <v>-0.03880962490593891</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.4667893949817093</v>
+        <v>-0.2165676912210912</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -2167,25 +2167,25 @@
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>0.417684068809007</v>
+        <v>0.8888758201271137</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>-0.02508747765506329</v>
+        <v>-0.162160455937545</v>
       </c>
       <c r="O4" t="n">
-        <v>-0.5132373770722745</v>
+        <v>-0.3014665486293167</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -2194,46 +2194,46 @@
         <v>-0</v>
       </c>
       <c r="T4" t="n">
-        <v>0.08355225222456056</v>
+        <v>0.1920707444627073</v>
       </c>
       <c r="U4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="V4" t="n">
         <v>0</v>
       </c>
       <c r="W4" t="n">
-        <v>-0.01937822669010482</v>
+        <v>-0.1943814002763433</v>
       </c>
       <c r="X4" t="n">
-        <v>0.002658846508433222</v>
+        <v>-0.01481640218773005</v>
       </c>
       <c r="Y4" t="n">
         <v>-0</v>
       </c>
       <c r="Z4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AA4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AB4" t="n">
         <v>-0</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.05032154152566831</v>
+        <v>0.02915931079150896</v>
       </c>
       <c r="AD4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AE4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AF4" t="n">
-        <v>0.0452238122739473</v>
+        <v>-0.4325883087767034</v>
       </c>
       <c r="AG4" t="n">
-        <v>-0.0006138402386187273</v>
+        <v>-0.177116916761541</v>
       </c>
       <c r="AH4" t="n">
         <v>-0</v>
@@ -2242,28 +2242,28 @@
         <v>-0</v>
       </c>
       <c r="AJ4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AK4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AL4" t="n">
-        <v>0.04783611672034568</v>
+        <v>0.07100156034737894</v>
       </c>
       <c r="AM4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
       </c>
       <c r="AO4" t="n">
-        <v>0.01105260176864441</v>
+        <v>-0.08751197442812333</v>
       </c>
       <c r="AP4" t="n">
-        <v>-0.09245244625987968</v>
+        <v>-0.02977348530376467</v>
       </c>
       <c r="AQ4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AR4" t="n">
         <v>-0</v>
@@ -2272,28 +2272,28 @@
         <v>0</v>
       </c>
       <c r="AT4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AU4" t="n">
-        <v>0.4422955460039922</v>
+        <v>0.8999644060588265</v>
       </c>
       <c r="AV4" t="n">
         <v>-0</v>
       </c>
       <c r="AW4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AX4" t="n">
-        <v>0.02909958576290571</v>
+        <v>-0.1899572132058835</v>
       </c>
       <c r="AY4" t="n">
-        <v>-0.3422947096666415</v>
+        <v>-0.2877109438313255</v>
       </c>
       <c r="AZ4" t="n">
         <v>0</v>
       </c>
       <c r="BA4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BB4" t="n">
         <v>0</v>
@@ -2302,34 +2302,34 @@
         <v>0</v>
       </c>
       <c r="BD4" t="n">
-        <v>0.1729184930104705</v>
+        <v>-0.005223259764982567</v>
       </c>
       <c r="BE4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BF4" t="n">
         <v>0</v>
       </c>
       <c r="BG4" t="n">
-        <v>-0.1709748528180153</v>
+        <v>-0.2153987441247562</v>
       </c>
       <c r="BH4" t="n">
-        <v>-0.205773175343103</v>
+        <v>-0.03537888606564646</v>
       </c>
       <c r="BI4" t="n">
         <v>0</v>
       </c>
       <c r="BJ4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BK4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BL4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BM4" t="n">
-        <v>0.2002558661155981</v>
+        <v>0.1625552795285686</v>
       </c>
       <c r="BN4" t="n">
         <v>0</v>
@@ -2338,16 +2338,16 @@
         <v>-0</v>
       </c>
       <c r="BP4" t="n">
-        <v>0.1039353742559497</v>
+        <v>0.1334187614211437</v>
       </c>
       <c r="BQ4" t="n">
-        <v>-0.002745880478777002</v>
+        <v>-0.06333506881801695</v>
       </c>
       <c r="BR4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BS4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BT4" t="n">
         <v>0</v>
@@ -2356,19 +2356,19 @@
         <v>-0</v>
       </c>
       <c r="BV4" t="n">
-        <v>0.2202303488753476</v>
+        <v>0.5756790283571528</v>
       </c>
       <c r="BW4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BX4" t="n">
         <v>0</v>
       </c>
       <c r="BY4" t="n">
-        <v>-0.02337664209677967</v>
+        <v>-0.0938506414998475</v>
       </c>
       <c r="BZ4" t="n">
-        <v>-0.1318044597539551</v>
+        <v>-0.1261243686077028</v>
       </c>
       <c r="CA4" t="n">
         <v>-0</v>
@@ -2380,10 +2380,10 @@
         <v>0</v>
       </c>
       <c r="CD4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="CE4" t="n">
-        <v>-0.1021583914261066</v>
+        <v>-0.1877970269757799</v>
       </c>
       <c r="CF4" t="n">
         <v>0</v>
@@ -2392,40 +2392,40 @@
         <v>-0</v>
       </c>
       <c r="CH4" t="n">
-        <v>-0.03532466201889423</v>
+        <v>0.07072009622528989</v>
       </c>
       <c r="CI4" t="n">
-        <v>0.08458899011131685</v>
+        <v>0.1182252210332908</v>
       </c>
       <c r="CJ4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CK4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="CL4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="CM4" t="n">
         <v>0</v>
       </c>
       <c r="CN4" t="n">
-        <v>-0.07622266115666991</v>
+        <v>-0.5349070891209067</v>
       </c>
       <c r="CO4" t="n">
         <v>-0</v>
       </c>
       <c r="CP4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="CQ4" t="n">
-        <v>0.0557340921369089</v>
+        <v>0.2613966506117856</v>
       </c>
       <c r="CR4" t="n">
-        <v>-0.008414755707959833</v>
+        <v>0.1436572325526864</v>
       </c>
       <c r="CS4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CT4" t="n">
         <v>-0</v>
@@ -2434,10 +2434,10 @@
         <v>-0</v>
       </c>
       <c r="CV4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CW4" t="n">
-        <v>-0.07580754175083776</v>
+        <v>-0.1837415808611344</v>
       </c>
       <c r="CX4" t="n">
         <v>-0</v>
@@ -2446,16 +2446,16 @@
         <v>0</v>
       </c>
       <c r="CZ4" t="n">
-        <v>-0.02465610247676257</v>
+        <v>0.01415621034023193</v>
       </c>
       <c r="DA4" t="n">
-        <v>0.08176320215717549</v>
+        <v>0.1203172450526309</v>
       </c>
       <c r="DB4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="DC4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DD4" t="n">
         <v>0</v>
@@ -2464,19 +2464,19 @@
         <v>-0</v>
       </c>
       <c r="DF4" t="n">
-        <v>-0.1214138544860826</v>
+        <v>-0.01548987196528341</v>
       </c>
       <c r="DG4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DH4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DI4" t="n">
-        <v>0.05060995353399975</v>
+        <v>-0.3361774532384811</v>
       </c>
       <c r="DJ4" t="n">
-        <v>0.007237652848752282</v>
+        <v>-0.07234625705639779</v>
       </c>
       <c r="DK4" t="n">
         <v>0</v>
@@ -2485,52 +2485,52 @@
         <v>0</v>
       </c>
       <c r="DM4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="DN4" t="n">
         <v>-0</v>
       </c>
       <c r="DO4" t="n">
-        <v>-0.04239344016925617</v>
+        <v>-0.1961143727728041</v>
       </c>
       <c r="DP4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="DQ4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DR4" t="n">
-        <v>0.0009569524015280327</v>
+        <v>0.1601952295190031</v>
       </c>
       <c r="DS4" t="n">
-        <v>0.01339061053045242</v>
+        <v>0.008637814132485554</v>
       </c>
       <c r="DT4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DU4" t="n">
         <v>-0</v>
       </c>
       <c r="DV4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="DW4" t="n">
         <v>-0</v>
       </c>
       <c r="DX4" t="n">
-        <v>0.04107505515408476</v>
+        <v>0.02111319435408945</v>
       </c>
       <c r="DY4" t="n">
         <v>0</v>
       </c>
       <c r="DZ4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EA4" t="n">
-        <v>-0.01863605066313381</v>
+        <v>0.2111101787924141</v>
       </c>
       <c r="EB4" t="n">
-        <v>-0.007276819296266104</v>
+        <v>-0.1987076781484413</v>
       </c>
       <c r="EC4" t="n">
         <v>-0</v>
@@ -2542,25 +2542,25 @@
         <v>-0</v>
       </c>
       <c r="EF4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EG4" t="n">
-        <v>-0.04617767171618136</v>
+        <v>-0.0003812455635604469</v>
       </c>
       <c r="EH4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EI4" t="n">
         <v>0</v>
       </c>
       <c r="EJ4" t="n">
-        <v>-0.0003742366308802584</v>
+        <v>-0.08326424169214684</v>
       </c>
       <c r="EK4" t="n">
-        <v>0.06937071822897516</v>
+        <v>0.07005540656746991</v>
       </c>
       <c r="EL4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EM4" t="n">
         <v>-0</v>
@@ -2569,10 +2569,10 @@
         <v>-0</v>
       </c>
       <c r="EO4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EP4" t="n">
-        <v>-0.03578639701946226</v>
+        <v>0.06901766726315298</v>
       </c>
       <c r="EQ4" t="n">
         <v>0</v>
@@ -2581,10 +2581,10 @@
         <v>-0</v>
       </c>
       <c r="ES4" t="n">
-        <v>-0.002511782053140976</v>
+        <v>-0.1008289781629941</v>
       </c>
       <c r="ET4" t="n">
-        <v>0.01378986376957782</v>
+        <v>0.06916514146792992</v>
       </c>
       <c r="EU4" t="n">
         <v>-0</v>
@@ -2593,13 +2593,13 @@
         <v>0</v>
       </c>
       <c r="EW4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EX4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EY4" t="n">
-        <v>-0.07548832889363698</v>
+        <v>-0.2103276517476383</v>
       </c>
       <c r="EZ4" t="n">
         <v>0</v>
@@ -2608,25 +2608,25 @@
         <v>-0</v>
       </c>
       <c r="FB4" t="n">
-        <v>-0.007989336884898357</v>
+        <v>0.007225353350047363</v>
       </c>
       <c r="FC4" t="n">
-        <v>0.08253256689453026</v>
+        <v>0.1204409276804921</v>
       </c>
       <c r="FD4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FE4" t="n">
         <v>0</v>
       </c>
       <c r="FF4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="FG4" t="n">
         <v>0</v>
       </c>
       <c r="FH4" t="n">
-        <v>-0.02667509012319998</v>
+        <v>-0.2622215421380676</v>
       </c>
       <c r="FI4" t="n">
         <v>-0</v>
@@ -2635,25 +2635,25 @@
         <v>-0</v>
       </c>
       <c r="FK4" t="n">
-        <v>-0.03698981378461119</v>
+        <v>0.2496844999611798</v>
       </c>
       <c r="FL4" t="n">
-        <v>0.1252882643213336</v>
+        <v>0.02027647527075637</v>
       </c>
       <c r="FM4" t="n">
         <v>0</v>
       </c>
       <c r="FN4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FO4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="FP4" t="n">
         <v>0</v>
       </c>
       <c r="FQ4" t="n">
-        <v>-0.003006450450050371</v>
+        <v>0.06000953316141198</v>
       </c>
       <c r="FR4" t="n">
         <v>-0</v>
@@ -2662,37 +2662,37 @@
         <v>-0</v>
       </c>
       <c r="FT4" t="n">
-        <v>-0.07167172005777364</v>
+        <v>-0.07758732239638148</v>
       </c>
       <c r="FU4" t="n">
-        <v>0.08244596212143086</v>
+        <v>-0.1283755579371373</v>
       </c>
       <c r="FV4" t="n">
         <v>-0</v>
       </c>
       <c r="FW4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FX4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="FY4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FZ4" t="n">
-        <v>-0.04856345833787983</v>
+        <v>-2.288541360379644e-05</v>
       </c>
       <c r="GA4" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="GB4" t="n">
         <v>-0</v>
       </c>
       <c r="GC4" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="GD4" t="n">
-        <v>-0.09574389797521202</v>
+        <v>-0.002258283347948613</v>
       </c>
       <c r="GE4" t="n">
         <v>-0</v>
@@ -2706,82 +2706,82 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.3215455388035593</v>
+        <v>-0.4531832812081955</v>
       </c>
       <c r="C5" t="n">
         <v>-0</v>
       </c>
       <c r="D5" t="n">
-        <v>0.4268003676076384</v>
+        <v>0.4837608259379137</v>
       </c>
       <c r="E5" t="n">
-        <v>0.04173892244839422</v>
+        <v>0.3168489085064923</v>
       </c>
       <c r="F5" t="n">
         <v>-0</v>
       </c>
       <c r="G5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.2718347124616217</v>
+        <v>-0.5024710680868091</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="M5" t="n">
-        <v>0.3772290778366779</v>
+        <v>0.6577634221555146</v>
       </c>
       <c r="N5" t="n">
-        <v>0.1040416034487176</v>
+        <v>0.4805985969219609</v>
       </c>
       <c r="O5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="R5" t="n">
         <v>-0</v>
       </c>
       <c r="S5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="T5" t="n">
-        <v>-0.05004081533165394</v>
+        <v>-0.07644077401021288</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
       </c>
       <c r="V5" t="n">
-        <v>0.1090151972643475</v>
+        <v>0.08424555629939109</v>
       </c>
       <c r="W5" t="n">
-        <v>0.1506715327024163</v>
+        <v>0.03274160387450207</v>
       </c>
       <c r="X5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Y5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Z5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA5" t="n">
         <v>-0</v>
@@ -2790,43 +2790,43 @@
         <v>-0</v>
       </c>
       <c r="AC5" t="n">
-        <v>-0.02887431776891015</v>
+        <v>0.005730420394870558</v>
       </c>
       <c r="AD5" t="n">
         <v>-0</v>
       </c>
       <c r="AE5" t="n">
-        <v>0.03099607481832935</v>
+        <v>-0.0161548377051621</v>
       </c>
       <c r="AF5" t="n">
-        <v>-0.002171664272443816</v>
+        <v>-0.100147824757869</v>
       </c>
       <c r="AG5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AH5" t="n">
         <v>0</v>
       </c>
       <c r="AI5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AJ5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AK5" t="n">
         <v>0</v>
       </c>
       <c r="AL5" t="n">
-        <v>-0.0539421869878648</v>
+        <v>-0.1996210686626445</v>
       </c>
       <c r="AM5" t="n">
         <v>-0</v>
       </c>
       <c r="AN5" t="n">
-        <v>0.03142291941106781</v>
+        <v>0.03266718695219852</v>
       </c>
       <c r="AO5" t="n">
-        <v>0.02255053611939785</v>
+        <v>-0.1979816155410517</v>
       </c>
       <c r="AP5" t="n">
         <v>-0</v>
@@ -2844,43 +2844,43 @@
         <v>0</v>
       </c>
       <c r="AU5" t="n">
-        <v>-0.4019385659229635</v>
+        <v>-0.5774974535069796</v>
       </c>
       <c r="AV5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AW5" t="n">
-        <v>0.06897792228284406</v>
+        <v>0.09699505135435685</v>
       </c>
       <c r="AX5" t="n">
-        <v>-0.1281272531239209</v>
+        <v>0.2495775368474911</v>
       </c>
       <c r="AY5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AZ5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BA5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BB5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BC5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BD5" t="n">
-        <v>-0.02430147668617014</v>
+        <v>0.05949699014797669</v>
       </c>
       <c r="BE5" t="n">
         <v>-0</v>
       </c>
       <c r="BF5" t="n">
-        <v>0.1903385692718083</v>
+        <v>0.2126817940117039</v>
       </c>
       <c r="BG5" t="n">
-        <v>0.2738649758045769</v>
+        <v>0.2492155149044933</v>
       </c>
       <c r="BH5" t="n">
         <v>-0</v>
@@ -2889,7 +2889,7 @@
         <v>0</v>
       </c>
       <c r="BJ5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BK5" t="n">
         <v>-0</v>
@@ -2898,19 +2898,19 @@
         <v>0</v>
       </c>
       <c r="BM5" t="n">
-        <v>-0.03628727823673479</v>
+        <v>0.0894868880036527</v>
       </c>
       <c r="BN5" t="n">
         <v>0</v>
       </c>
       <c r="BO5" t="n">
-        <v>-0.001377243529933103</v>
+        <v>-0.08749210577363288</v>
       </c>
       <c r="BP5" t="n">
-        <v>-0.08873255418709254</v>
+        <v>-0.04476900226085904</v>
       </c>
       <c r="BQ5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BR5" t="n">
         <v>0</v>
@@ -2925,46 +2925,46 @@
         <v>0</v>
       </c>
       <c r="BV5" t="n">
-        <v>-0.2477178503924696</v>
+        <v>-0.4344969099678129</v>
       </c>
       <c r="BW5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BX5" t="n">
-        <v>0.05550396287344841</v>
+        <v>0.2815807230769858</v>
       </c>
       <c r="BY5" t="n">
-        <v>-0.004352928206524021</v>
+        <v>0.1000106632888934</v>
       </c>
       <c r="BZ5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="CA5" t="n">
         <v>-0</v>
       </c>
       <c r="CB5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="CC5" t="n">
         <v>-0</v>
       </c>
       <c r="CD5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="CE5" t="n">
-        <v>0.08573867346287942</v>
+        <v>0.2864744914409602</v>
       </c>
       <c r="CF5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CG5" t="n">
-        <v>-0.09433899030873051</v>
+        <v>-0.1694479530507532</v>
       </c>
       <c r="CH5" t="n">
-        <v>0.0242901099866377</v>
+        <v>-0.01999625383159155</v>
       </c>
       <c r="CI5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CJ5" t="n">
         <v>0</v>
@@ -2979,19 +2979,19 @@
         <v>-0</v>
       </c>
       <c r="CN5" t="n">
-        <v>-0.02291582543317137</v>
+        <v>0.2280260382961562</v>
       </c>
       <c r="CO5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CP5" t="n">
-        <v>0.04344608758541615</v>
+        <v>-0.3669643868573721</v>
       </c>
       <c r="CQ5" t="n">
-        <v>-0.0102587016080173</v>
+        <v>-0.1328837451241059</v>
       </c>
       <c r="CR5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CS5" t="n">
         <v>0</v>
@@ -3000,22 +3000,22 @@
         <v>0</v>
       </c>
       <c r="CU5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="CV5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CW5" t="n">
-        <v>0.08070271466793195</v>
+        <v>0.274744490258868</v>
       </c>
       <c r="CX5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="CY5" t="n">
-        <v>-0.09078368292945241</v>
+        <v>-0.1901359838881012</v>
       </c>
       <c r="CZ5" t="n">
-        <v>-0.007199192679304272</v>
+        <v>-0.05261814035989516</v>
       </c>
       <c r="DA5" t="n">
         <v>-0</v>
@@ -3030,22 +3030,22 @@
         <v>-0</v>
       </c>
       <c r="DE5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="DF5" t="n">
-        <v>0.007633889506394685</v>
+        <v>0.005382956578433446</v>
       </c>
       <c r="DG5" t="n">
         <v>0</v>
       </c>
       <c r="DH5" t="n">
-        <v>-0.04186968986327556</v>
+        <v>-0.07210540266974642</v>
       </c>
       <c r="DI5" t="n">
-        <v>-0.0798733474127364</v>
+        <v>0.07976195286211725</v>
       </c>
       <c r="DJ5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DK5" t="n">
         <v>0</v>
@@ -3057,25 +3057,25 @@
         <v>-0</v>
       </c>
       <c r="DN5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="DO5" t="n">
-        <v>0.06040769406593899</v>
+        <v>0.1069822892894526</v>
       </c>
       <c r="DP5" t="n">
         <v>0</v>
       </c>
       <c r="DQ5" t="n">
-        <v>-0.1282058627817134</v>
+        <v>-0.1330042773840573</v>
       </c>
       <c r="DR5" t="n">
-        <v>0.003082269080396409</v>
+        <v>0.05259537213572242</v>
       </c>
       <c r="DS5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DT5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DU5" t="n">
         <v>0</v>
@@ -3084,46 +3084,46 @@
         <v>-0</v>
       </c>
       <c r="DW5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DX5" t="n">
-        <v>-0.01187928681479571</v>
+        <v>-0.06280648897785196</v>
       </c>
       <c r="DY5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DZ5" t="n">
-        <v>0.007776695515561097</v>
+        <v>-0.04664092751532871</v>
       </c>
       <c r="EA5" t="n">
-        <v>0.01436470848984942</v>
+        <v>-0.09587447513027886</v>
       </c>
       <c r="EB5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EC5" t="n">
         <v>0</v>
       </c>
       <c r="ED5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EE5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EF5" t="n">
         <v>-0</v>
       </c>
       <c r="EG5" t="n">
-        <v>0.008623267379450121</v>
+        <v>0.2380334424395218</v>
       </c>
       <c r="EH5" t="n">
         <v>-0</v>
       </c>
       <c r="EI5" t="n">
-        <v>-0.03287586678445679</v>
+        <v>-0.07562141415390744</v>
       </c>
       <c r="EJ5" t="n">
-        <v>-0.02019692815802627</v>
+        <v>-0.119961558994652</v>
       </c>
       <c r="EK5" t="n">
         <v>0</v>
@@ -3132,31 +3132,31 @@
         <v>0</v>
       </c>
       <c r="EM5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EN5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EO5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EP5" t="n">
-        <v>0.08328260824759384</v>
+        <v>0.2151974317109577</v>
       </c>
       <c r="EQ5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="ER5" t="n">
-        <v>-0.06429325396644589</v>
+        <v>-0.1472405031280093</v>
       </c>
       <c r="ES5" t="n">
-        <v>0.06278479355845612</v>
+        <v>-0.05650369024290513</v>
       </c>
       <c r="ET5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EU5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EV5" t="n">
         <v>-0</v>
@@ -3165,19 +3165,19 @@
         <v>0</v>
       </c>
       <c r="EX5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EY5" t="n">
-        <v>0.08903957109298768</v>
+        <v>0.3169804486597755</v>
       </c>
       <c r="EZ5" t="n">
         <v>0</v>
       </c>
       <c r="FA5" t="n">
-        <v>-0.09463752330257852</v>
+        <v>-0.2297463173006575</v>
       </c>
       <c r="FB5" t="n">
-        <v>0.01800727865349654</v>
+        <v>-0.04668581551134547</v>
       </c>
       <c r="FC5" t="n">
         <v>0</v>
@@ -3189,31 +3189,31 @@
         <v>-0</v>
       </c>
       <c r="FF5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FG5" t="n">
         <v>0</v>
       </c>
       <c r="FH5" t="n">
-        <v>0.0414521633608991</v>
+        <v>0.1636906759610375</v>
       </c>
       <c r="FI5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FJ5" t="n">
-        <v>0.04354840130687807</v>
+        <v>0.1627733883853974</v>
       </c>
       <c r="FK5" t="n">
-        <v>-0.03291359847804542</v>
+        <v>-0.05590803395578389</v>
       </c>
       <c r="FL5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="FM5" t="n">
         <v>0</v>
       </c>
       <c r="FN5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FO5" t="n">
         <v>0</v>
@@ -3222,16 +3222,16 @@
         <v>0</v>
       </c>
       <c r="FQ5" t="n">
-        <v>-0.01221464163930013</v>
+        <v>-0.1994396429015716</v>
       </c>
       <c r="FR5" t="n">
         <v>0</v>
       </c>
       <c r="FS5" t="n">
-        <v>0.02831107797667131</v>
+        <v>-0.1246075097004791</v>
       </c>
       <c r="FT5" t="n">
-        <v>-0.01839111089489138</v>
+        <v>-0.003619124464162399</v>
       </c>
       <c r="FU5" t="n">
         <v>0</v>
@@ -3240,22 +3240,22 @@
         <v>0</v>
       </c>
       <c r="FW5" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FX5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="FY5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="FZ5" t="n">
-        <v>0.06933134074777453</v>
+        <v>0.1794520301620204</v>
       </c>
       <c r="GA5" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="GB5" t="n">
-        <v>0.06106598869935288</v>
+        <v>-0.1186795538729922</v>
       </c>
       <c r="GC5" t="n">
         <v>-0</v>
@@ -3275,19 +3275,19 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="B6" t="n">
-        <v>-0.4984606456358585</v>
+        <v>-0.4967447287547417</v>
       </c>
       <c r="C6" t="n">
         <v>-0</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1630556590172297</v>
+        <v>0.4703860228028513</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1726498722410141</v>
+        <v>0.07931035731583583</v>
       </c>
       <c r="F6" t="n">
         <v>-0</v>
@@ -3305,16 +3305,16 @@
         <v>-0</v>
       </c>
       <c r="K6" t="n">
-        <v>-0.3279555481603417</v>
+        <v>-0.4632402570887008</v>
       </c>
       <c r="L6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="M6" t="n">
-        <v>0.1702610439958268</v>
+        <v>0.6546953481082753</v>
       </c>
       <c r="N6" t="n">
-        <v>0.09870378554691323</v>
+        <v>0.1207738151519414</v>
       </c>
       <c r="O6" t="n">
         <v>-0</v>
@@ -3329,46 +3329,46 @@
         <v>-0</v>
       </c>
       <c r="S6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="T6" t="n">
-        <v>-0.04977107854097373</v>
+        <v>-0.01924964972915242</v>
       </c>
       <c r="U6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="V6" t="n">
-        <v>0.07105694791705165</v>
+        <v>0.05746259285113228</v>
       </c>
       <c r="W6" t="n">
-        <v>0.1314246000310552</v>
+        <v>0.03126227931293323</v>
       </c>
       <c r="X6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="Y6" t="n">
         <v>-0</v>
       </c>
       <c r="Z6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AA6" t="n">
         <v>-0</v>
       </c>
       <c r="AB6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AC6" t="n">
-        <v>-0.008674013499658548</v>
+        <v>-0.01545113800665792</v>
       </c>
       <c r="AD6" t="n">
         <v>-0</v>
       </c>
       <c r="AE6" t="n">
-        <v>0.1101794412399949</v>
+        <v>0.1407706950396675</v>
       </c>
       <c r="AF6" t="n">
-        <v>0.02797574269990794</v>
+        <v>-0.168073011833145</v>
       </c>
       <c r="AG6" t="n">
         <v>0</v>
@@ -3377,25 +3377,25 @@
         <v>-0</v>
       </c>
       <c r="AI6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AJ6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AK6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AL6" t="n">
-        <v>-0.06945021309965831</v>
+        <v>-0.1843193915870669</v>
       </c>
       <c r="AM6" t="n">
         <v>-0</v>
       </c>
       <c r="AN6" t="n">
-        <v>0.01504631513886189</v>
+        <v>0.06962824870048588</v>
       </c>
       <c r="AO6" t="n">
-        <v>0.08275532588214642</v>
+        <v>-0.2472024355181901</v>
       </c>
       <c r="AP6" t="n">
         <v>-0</v>
@@ -3413,22 +3413,22 @@
         <v>0</v>
       </c>
       <c r="AU6" t="n">
-        <v>-0.2217662334140048</v>
+        <v>-0.2938530699010106</v>
       </c>
       <c r="AV6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AW6" t="n">
-        <v>0.09189041611866648</v>
+        <v>0.2402350319047131</v>
       </c>
       <c r="AX6" t="n">
-        <v>0.1593328705998186</v>
+        <v>0.1164195965981216</v>
       </c>
       <c r="AY6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AZ6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BA6" t="n">
         <v>-0</v>
@@ -3437,52 +3437,52 @@
         <v>-0</v>
       </c>
       <c r="BC6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BD6" t="n">
-        <v>-0.1701912849948955</v>
+        <v>0.04532219281538906</v>
       </c>
       <c r="BE6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BF6" t="n">
-        <v>0.1496924177117338</v>
+        <v>0.0817351347888019</v>
       </c>
       <c r="BG6" t="n">
-        <v>0.1637932605620342</v>
+        <v>0.104446135131501</v>
       </c>
       <c r="BH6" t="n">
         <v>-0</v>
       </c>
       <c r="BI6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BJ6" t="n">
         <v>0</v>
       </c>
       <c r="BK6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BL6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BM6" t="n">
-        <v>-0.01750633267065132</v>
+        <v>0.1583519945794504</v>
       </c>
       <c r="BN6" t="n">
         <v>0</v>
       </c>
       <c r="BO6" t="n">
-        <v>0.02805024861406306</v>
+        <v>-0.04052267095353973</v>
       </c>
       <c r="BP6" t="n">
-        <v>-0.0150707712974798</v>
+        <v>0.03438608857713858</v>
       </c>
       <c r="BQ6" t="n">
         <v>0</v>
       </c>
       <c r="BR6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BS6" t="n">
         <v>0</v>
@@ -3491,19 +3491,19 @@
         <v>0</v>
       </c>
       <c r="BU6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="BV6" t="n">
-        <v>-0.1869627900357449</v>
+        <v>-0.2508366729377684</v>
       </c>
       <c r="BW6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="BX6" t="n">
-        <v>0.08269522822173711</v>
+        <v>0.1920874656493603</v>
       </c>
       <c r="BY6" t="n">
-        <v>0.07160141034564049</v>
+        <v>-0.004928790616186646</v>
       </c>
       <c r="BZ6" t="n">
         <v>-0</v>
@@ -3521,22 +3521,22 @@
         <v>-0</v>
       </c>
       <c r="CE6" t="n">
-        <v>0.07314132801364766</v>
+        <v>0.2258789395106455</v>
       </c>
       <c r="CF6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CG6" t="n">
-        <v>-0.04829610327900825</v>
+        <v>-0.1437682519042735</v>
       </c>
       <c r="CH6" t="n">
-        <v>0.0220016211943641</v>
+        <v>0.0350637053571804</v>
       </c>
       <c r="CI6" t="n">
         <v>0</v>
       </c>
       <c r="CJ6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CK6" t="n">
         <v>-0</v>
@@ -3548,19 +3548,19 @@
         <v>-0</v>
       </c>
       <c r="CN6" t="n">
-        <v>-0.07464434621248818</v>
+        <v>0.09343133718128831</v>
       </c>
       <c r="CO6" t="n">
         <v>0</v>
       </c>
       <c r="CP6" t="n">
-        <v>-0.1890121403656911</v>
+        <v>-0.2379759972864895</v>
       </c>
       <c r="CQ6" t="n">
-        <v>-0.0002884619474195425</v>
+        <v>-0.1171308587482566</v>
       </c>
       <c r="CR6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CS6" t="n">
         <v>0</v>
@@ -3569,22 +3569,22 @@
         <v>-0</v>
       </c>
       <c r="CU6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="CV6" t="n">
         <v>0</v>
       </c>
       <c r="CW6" t="n">
-        <v>0.08217006691740611</v>
+        <v>0.2361100071935326</v>
       </c>
       <c r="CX6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="CY6" t="n">
-        <v>-0.03760318759258864</v>
+        <v>-0.1569364090107236</v>
       </c>
       <c r="CZ6" t="n">
-        <v>0.006921899711900212</v>
+        <v>0.005021504899417766</v>
       </c>
       <c r="DA6" t="n">
         <v>-0</v>
@@ -3602,16 +3602,16 @@
         <v>-0</v>
       </c>
       <c r="DF6" t="n">
-        <v>0.1409288196047623</v>
+        <v>0.09291384842058308</v>
       </c>
       <c r="DG6" t="n">
         <v>0</v>
       </c>
       <c r="DH6" t="n">
-        <v>-0.06822517556188347</v>
+        <v>-0.07721758768425871</v>
       </c>
       <c r="DI6" t="n">
-        <v>-0.005384569511356482</v>
+        <v>0.03068283112069992</v>
       </c>
       <c r="DJ6" t="n">
         <v>0</v>
@@ -3623,25 +3623,25 @@
         <v>-0</v>
       </c>
       <c r="DM6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DN6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="DO6" t="n">
-        <v>0.007838807386637002</v>
+        <v>0.1088648026341609</v>
       </c>
       <c r="DP6" t="n">
         <v>0</v>
       </c>
       <c r="DQ6" t="n">
-        <v>-0.022049683320956</v>
+        <v>-0.08444229410637363</v>
       </c>
       <c r="DR6" t="n">
-        <v>-0.04447367122941184</v>
+        <v>0.05758920467558059</v>
       </c>
       <c r="DS6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DT6" t="n">
         <v>0</v>
@@ -3653,22 +3653,22 @@
         <v>-0</v>
       </c>
       <c r="DW6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="DX6" t="n">
-        <v>0.1093686026545412</v>
+        <v>0.06061771148596962</v>
       </c>
       <c r="DY6" t="n">
         <v>0</v>
       </c>
       <c r="DZ6" t="n">
-        <v>-0.0463918430016036</v>
+        <v>0.01137472661927157</v>
       </c>
       <c r="EA6" t="n">
-        <v>0.00413492236823502</v>
+        <v>-0.013285228916829</v>
       </c>
       <c r="EB6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="EC6" t="n">
         <v>0</v>
@@ -3683,49 +3683,49 @@
         <v>-0</v>
       </c>
       <c r="EG6" t="n">
-        <v>0.05744850113713924</v>
+        <v>0.2391866318360412</v>
       </c>
       <c r="EH6" t="n">
         <v>-0</v>
       </c>
       <c r="EI6" t="n">
-        <v>0.05538835150769398</v>
+        <v>-0.1156661667629101</v>
       </c>
       <c r="EJ6" t="n">
-        <v>0.06456316018268303</v>
+        <v>-0.03179647219976433</v>
       </c>
       <c r="EK6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EL6" t="n">
         <v>-0</v>
       </c>
       <c r="EM6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EN6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EO6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EP6" t="n">
-        <v>0.02534774737078672</v>
+        <v>0.1637315641077234</v>
       </c>
       <c r="EQ6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="ER6" t="n">
-        <v>-0.05251768604493646</v>
+        <v>-0.09266773936223631</v>
       </c>
       <c r="ES6" t="n">
-        <v>-0.002826237861208346</v>
+        <v>-0.07411087057056909</v>
       </c>
       <c r="ET6" t="n">
         <v>0</v>
       </c>
       <c r="EU6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="EV6" t="n">
         <v>-0</v>
@@ -3737,73 +3737,73 @@
         <v>-0</v>
       </c>
       <c r="EY6" t="n">
-        <v>0.08255266764086829</v>
+        <v>0.2596140822925206</v>
       </c>
       <c r="EZ6" t="n">
         <v>0</v>
       </c>
       <c r="FA6" t="n">
-        <v>-0.02979239188072513</v>
+        <v>-0.18217927923712</v>
       </c>
       <c r="FB6" t="n">
-        <v>0.02332877836078678</v>
+        <v>0.01939002663553602</v>
       </c>
       <c r="FC6" t="n">
         <v>0</v>
       </c>
       <c r="FD6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="FE6" t="n">
         <v>-0</v>
       </c>
       <c r="FF6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FG6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FH6" t="n">
-        <v>-0.04531463150076858</v>
+        <v>-0.09337689124888997</v>
       </c>
       <c r="FI6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FJ6" t="n">
-        <v>0.04543308323280197</v>
+        <v>0.1750441343891178</v>
       </c>
       <c r="FK6" t="n">
-        <v>-0.0177003039992163</v>
+        <v>-0.1912235224561148</v>
       </c>
       <c r="FL6" t="n">
         <v>0</v>
       </c>
       <c r="FM6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FN6" t="n">
         <v>0</v>
       </c>
       <c r="FO6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="FP6" t="n">
         <v>-0</v>
       </c>
       <c r="FQ6" t="n">
-        <v>0.1238616740461258</v>
+        <v>0.1644657810984315</v>
       </c>
       <c r="FR6" t="n">
         <v>0</v>
       </c>
       <c r="FS6" t="n">
-        <v>-0.08138835912372706</v>
+        <v>-0.01673281538376196</v>
       </c>
       <c r="FT6" t="n">
-        <v>-0.1981051395525977</v>
+        <v>-0.3075993929965953</v>
       </c>
       <c r="FU6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="FV6" t="n">
         <v>-0</v>
@@ -3818,25 +3818,25 @@
         <v>-0</v>
       </c>
       <c r="FZ6" t="n">
-        <v>-0.008877747759138481</v>
+        <v>0.2239425198180413</v>
       </c>
       <c r="GA6" t="n">
         <v>0</v>
       </c>
       <c r="GB6" t="n">
-        <v>0.01675310711426355</v>
+        <v>-0.07037003541547156</v>
       </c>
       <c r="GC6" t="n">
         <v>-0</v>
       </c>
       <c r="GD6" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="GE6" t="n">
         <v>0</v>
       </c>
       <c r="GF6" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="GG6" t="n">
         <v>-0</v>

</xml_diff>